<commit_message>
fix(auth): update AuthPage layout and test cases document
</commit_message>
<xml_diff>
--- a/docs/test-cases-auth.xlsx
+++ b/docs/test-cases-auth.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\AIPETCLIENT\leBotChatClient\le-bot-frontend\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DDA052-AD66-4FAB-BC30-6D3675F6C1E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6592B496-B1FF-4271-A108-C34EE44D6ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="314">
   <si>
     <t>用例编号</t>
   </si>
@@ -1075,6 +1075,10 @@
   </si>
   <si>
     <t>无法测试，等手机测试</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>完成</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1711,7 +1715,9 @@
       <c r="G4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="5"/>
+      <c r="H4" s="15" t="s">
+        <v>313</v>
+      </c>
       <c r="I4" s="2" t="s">
         <v>18</v>
       </c>

</xml_diff>